<commit_message>
add .gitignore and requirements.txt files and clean up folders. modify script to save output in 'outputs' folder
</commit_message>
<xml_diff>
--- a/data/spreadsheets/nga_lga_pol_map.xlsx
+++ b/data/spreadsheets/nga_lga_pol_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jarretangbazo/nga_population_estimation/data/spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C08A03F-368E-4C4B-97E7-4A7AA25BF9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDD9386-0E82-0744-BE2A-1193767ECDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{A3DC1CEF-6063-2F4F-B8D4-B0FB9E426514}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="18440" xr2:uid="{A3DC1CEF-6063-2F4F-B8D4-B0FB9E426514}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -604,9 +604,6 @@
     <t>Kogi Central</t>
   </si>
   <si>
-    <t>Ajaokuta</t>
-  </si>
-  <si>
     <t>Adavi/Okehi</t>
   </si>
   <si>
@@ -868,9 +865,6 @@
     <t>Jigawa North East</t>
   </si>
   <si>
-    <t>Hadejia/Kafin Hausa</t>
-  </si>
-  <si>
     <t>Oru East/Orsu/Orlu</t>
   </si>
   <si>
@@ -1426,9 +1420,6 @@
     <t>Edo Central</t>
   </si>
   <si>
-    <t>Esan Central/Esan South/Igueben</t>
-  </si>
-  <si>
     <t>Esan North East/Esan South East</t>
   </si>
   <si>
@@ -1445,6 +1436,15 @@
   </si>
   <si>
     <t>Owan East/Owan West</t>
+  </si>
+  <si>
+    <t>Esan Central/Esan South/Igueben/Esan West</t>
+  </si>
+  <si>
+    <t>Hadejia/Kafin Hausa/Auyo</t>
+  </si>
+  <si>
+    <t>Ajaokuta/Kogi</t>
   </si>
 </sst>
 </file>
@@ -1826,1741 +1826,1741 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>431</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>427</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>429</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B8" s="1" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>420</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B13" s="1" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>413</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>409</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B20" s="1" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" s="1" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>404</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B24" s="1" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>400</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B27" s="1" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B28" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>396</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B30" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B32" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>391</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" s="1" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B34" s="1" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B36" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>386</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B39" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>382</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B40" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>382</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B41" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B42" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B43" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B44" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B45" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B48" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B49" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>376</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B50" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="C50" s="1" t="s">
         <v>376</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B51" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B52" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B53" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B54" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B55" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B56" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B57" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>371</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B58" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="C58" s="1" t="s">
         <v>371</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B59" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B60" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B61" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B62" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B63" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>367</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B64" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B65" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B66" s="1" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B67" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="C67" s="1" t="s">
         <v>362</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B68" s="1" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B69" s="1" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B70" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B71" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>357</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B72" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B73" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B74" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B75" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>352</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B76" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B77" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B78" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>348</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B79" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B80" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="81" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B81" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="C81" s="1" t="s">
         <v>344</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B82" s="1" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B83" s="1" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B84" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>340</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="85" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B85" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>340</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="86" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B86" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B87" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B88" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B89" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="90" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B90" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B91" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B92" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B93" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="94" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B94" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>333</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="95" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B95" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>333</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="96" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B96" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="97" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B97" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="98" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B98" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="99" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B99" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="100" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B100" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="101" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B101" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="102" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B102" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="103" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B103" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="104" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B104" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="105" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B105" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="106" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B106" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="107" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B107" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="108" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B108" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="109" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B109" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="110" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B110" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="111" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B111" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="112" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B112" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="113" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B113" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="114" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B114" s="1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="115" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B115" s="1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="116" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B116" s="1" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="117" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B117" s="1" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="118" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B118" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C118" s="1" t="s">
         <v>311</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="119" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B119" s="1" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="120" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B120" s="1" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="121" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B121" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C121" s="1" t="s">
         <v>307</v>
-      </c>
-      <c r="C121" s="1" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="122" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B122" s="1" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="123" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B123" s="1" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="124" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B124" s="1" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="125" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B125" s="1" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="126" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B126" s="1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="127" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B127" s="1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="128" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B128" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="129" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B129" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="130" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B130" s="1" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="131" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B131" s="1" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="132" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B132" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="133" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B133" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="134" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B134" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="135" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B135" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C135" s="1" t="s">
         <v>287</v>
-      </c>
-      <c r="C135" s="1" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="136" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B136" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="137" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B137" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="138" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B138" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="139" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B139" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="140" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B140" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="141" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B141" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C141" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="C141" s="1" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="142" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B142" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="143" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B143" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="144" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B144" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>277</v>
+        <v>468</v>
       </c>
     </row>
     <row r="145" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B145" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="146" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B146" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="147" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B147" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="148" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B148" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="C148" s="1" t="s">
         <v>271</v>
-      </c>
-      <c r="C148" s="1" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="149" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B149" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="150" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B150" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="151" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B151" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="152" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B152" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="153" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B153" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C153" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="C153" s="1" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="154" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B154" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="155" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B155" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="156" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B156" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="157" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B157" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C157" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="C157" s="1" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="158" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B158" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="159" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B159" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="160" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B160" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="161" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B161" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="162" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B162" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="163" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B163" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="164" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B164" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C164" s="1" t="s">
         <v>254</v>
-      </c>
-      <c r="C164" s="1" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="165" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B165" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="166" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B166" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="167" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B167" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="168" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B168" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="169" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B169" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C169" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="C169" s="1" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="170" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B170" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="171" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B171" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="172" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B172" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="173" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B173" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="174" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B174" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="175" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B175" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C175" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="176" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B176" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="177" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B177" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="178" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B178" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="179" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B179" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C179" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="180" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B180" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C180" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="C180" s="1" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="181" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B181" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="182" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B182" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="183" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B183" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C183" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="184" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B184" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C184" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="185" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B185" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C185" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="186" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B186" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C186" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="C186" s="1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="187" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B187" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C187" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="188" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B188" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C188" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="189" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B189" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C189" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="190" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B190" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="191" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B191" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C191" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="192" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B192" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C192" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="193" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B193" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C193" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="C193" s="1" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="194" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B194" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C194" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="195" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B195" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C195" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="196" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B196" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C196" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="197" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B197" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C197" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="198" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B198" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C198" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="C198" s="1" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="199" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B199" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C199" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="200" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B200" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="201" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B201" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C201" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="202" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B202" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="203" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B203" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C203" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="C203" s="1" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="204" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B204" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="205" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B205" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C205" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="206" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B206" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C206" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="207" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B207" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="208" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B208" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C208" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="C208" s="1" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="209" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B209" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C209" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="210" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B210" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C210" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="211" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B211" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C211" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="C211" s="1" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="212" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B212" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C212" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="213" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B213" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C213" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="214" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B214" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C214" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="C214" s="1" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="215" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B215" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C215" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="216" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B216" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C216" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="C216" s="1" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="217" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B217" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C217" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="218" spans="2:3" x14ac:dyDescent="0.2">
@@ -3568,7 +3568,7 @@
         <v>188</v>
       </c>
       <c r="C218" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="219" spans="2:3" x14ac:dyDescent="0.2">
@@ -3576,7 +3576,7 @@
         <v>188</v>
       </c>
       <c r="C219" s="1" t="s">
-        <v>189</v>
+        <v>469</v>
       </c>
     </row>
     <row r="220" spans="2:3" x14ac:dyDescent="0.2">
@@ -4733,194 +4733,194 @@
     </row>
     <row r="364" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B364" s="1" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="C364" s="1" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="365" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B365" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="C365" s="1" t="s">
         <v>437</v>
-      </c>
-      <c r="C365" s="1" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="366" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B366" s="1" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C366" s="1" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="367" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B367" s="1" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C367" s="1" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="368" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B368" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="C368" s="1" t="s">
         <v>442</v>
-      </c>
-      <c r="C368" s="1" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="369" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B369" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C369" s="1" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="370" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B370" s="1" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C370" s="1" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="371" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B371" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="C371" s="1" t="s">
         <v>447</v>
-      </c>
-      <c r="C371" s="1" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="372" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B372" s="1" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C372" s="1" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="373" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B373" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C373" s="1" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="374" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B374" s="1" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C374" s="1" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="375" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B375" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C375" s="1" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="376" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B376" s="1" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C376" s="1" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="377" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B377" s="1" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C377" s="1" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="378" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B378" s="1" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C378" s="1" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="379" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B379" s="1" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C379" s="1" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="380" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B380" s="1" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C380" s="1" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="381" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B381" s="1" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="C381" s="1" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
     </row>
     <row r="382" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B382" s="1" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="C382" s="1" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
     </row>
     <row r="383" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B383" s="1" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C383" s="1" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="384" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B384" s="1" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C384" s="1" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="385" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B385" s="1" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C385" s="1" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="386" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B386" s="1" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C386" s="1" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
     </row>
     <row r="387" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B387" s="1" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C387" s="1" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
     </row>
   </sheetData>

</xml_diff>